<commit_message>
GitHub Actions Results added
</commit_message>
<xml_diff>
--- a/Daily_Report/Top 7 broker List with its Turnover 2022-12-13.xlsx
+++ b/Daily_Report/Top 7 broker List with its Turnover 2022-12-13.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="256">
   <si>
     <t>Date: 2022-12-13</t>
   </si>
@@ -62,64 +62,61 @@
     <t>Naasa Securities Co. Ltd.</t>
   </si>
   <si>
-    <t>Sweta Securities Pvt. Limited</t>
-  </si>
-  <si>
     <t>Vision Securities Pvt.Limited</t>
   </si>
   <si>
     <t>Imperial Securities Co .Pvt.Limited</t>
   </si>
   <si>
-    <t>Neev Securities Pvt.Ltd</t>
-  </si>
-  <si>
-    <t>Sani Securities Company Limited</t>
-  </si>
-  <si>
-    <t>Dakshinkali Investment Securities Pvt.Limited</t>
+    <t>Online Securities Pvt.Ltd</t>
+  </si>
+  <si>
+    <t>Dynamic Money Managers Securities Pvt.Ltd</t>
+  </si>
+  <si>
+    <t>Trishul Securities And Investment Limited</t>
+  </si>
+  <si>
+    <t>Agrawal Securities Pvt. Limited</t>
   </si>
   <si>
     <t>58</t>
   </si>
   <si>
-    <t>25</t>
-  </si>
-  <si>
     <t>34</t>
   </si>
   <si>
     <t>45</t>
   </si>
   <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>193,015,380.7</t>
-  </si>
-  <si>
-    <t>75,091,543.2</t>
-  </si>
-  <si>
-    <t>65,912,758.8</t>
-  </si>
-  <si>
-    <t>58,602,254.6</t>
-  </si>
-  <si>
-    <t>54,993,984.5</t>
-  </si>
-  <si>
-    <t>41,874,722.4</t>
-  </si>
-  <si>
-    <t>40,090,942.9</t>
+    <t>49</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>97,134,358.52</t>
+  </si>
+  <si>
+    <t>50,928,481.1</t>
+  </si>
+  <si>
+    <t>43,104,606.3</t>
+  </si>
+  <si>
+    <t>28,636,146.33</t>
+  </si>
+  <si>
+    <t>25,294,118.5</t>
+  </si>
+  <si>
+    <t>21,746,190.1</t>
+  </si>
+  <si>
+    <t>21,432,847.1</t>
   </si>
   <si>
     <t>0.0</t>
@@ -140,322 +137,319 @@
     <t>% of turnover</t>
   </si>
   <si>
-    <t>KBLPO</t>
-  </si>
-  <si>
-    <t>51,000,000.0</t>
+    <t>NBL</t>
+  </si>
+  <si>
+    <t>30,364,354.3</t>
+  </si>
+  <si>
+    <t>NTC</t>
+  </si>
+  <si>
+    <t>13,785,110.5</t>
+  </si>
+  <si>
+    <t>NICA</t>
+  </si>
+  <si>
+    <t>10,442,876.0</t>
+  </si>
+  <si>
+    <t>NRIC</t>
+  </si>
+  <si>
+    <t>8,051,561.4</t>
+  </si>
+  <si>
+    <t>SMFDB</t>
+  </si>
+  <si>
+    <t>4,803,383.8</t>
+  </si>
+  <si>
+    <t>FMDBL</t>
+  </si>
+  <si>
+    <t>9,338,341.0</t>
+  </si>
+  <si>
+    <t>6,227,615.0</t>
+  </si>
+  <si>
+    <t>5,065,395.5</t>
+  </si>
+  <si>
+    <t>RIDI</t>
+  </si>
+  <si>
+    <t>4,588,646.0</t>
+  </si>
+  <si>
+    <t>CCBL</t>
+  </si>
+  <si>
+    <t>2,728,927.6</t>
+  </si>
+  <si>
+    <t>6,479,066.0</t>
+  </si>
+  <si>
+    <t>3,888,384.4</t>
+  </si>
+  <si>
+    <t>SHIVM</t>
+  </si>
+  <si>
+    <t>3,414,751.0</t>
   </si>
   <si>
     <t>NABIL</t>
   </si>
   <si>
-    <t>14,415,410.2</t>
-  </si>
-  <si>
-    <t>PRVU</t>
-  </si>
-  <si>
-    <t>14,152,720.8</t>
-  </si>
-  <si>
-    <t>NCCB</t>
-  </si>
-  <si>
-    <t>12,758,379.4</t>
-  </si>
-  <si>
-    <t>RIDI</t>
-  </si>
-  <si>
-    <t>9,796,502.5</t>
-  </si>
-  <si>
-    <t>ALBSLP</t>
-  </si>
-  <si>
-    <t>59,350,000.0</t>
-  </si>
-  <si>
-    <t>2,476,473.5</t>
+    <t>2,711,429.0</t>
+  </si>
+  <si>
+    <t>SAHAS</t>
+  </si>
+  <si>
+    <t>2,430,466.7</t>
+  </si>
+  <si>
+    <t>4,090,557.5</t>
+  </si>
+  <si>
+    <t>3,024,006.5</t>
+  </si>
+  <si>
+    <t>HDL</t>
+  </si>
+  <si>
+    <t>1,647,781.7</t>
+  </si>
+  <si>
+    <t>HEI</t>
+  </si>
+  <si>
+    <t>1,086,341.5</t>
+  </si>
+  <si>
+    <t>1,053,454.0</t>
+  </si>
+  <si>
+    <t>3,876,809.0</t>
+  </si>
+  <si>
+    <t>3,073,083.6</t>
+  </si>
+  <si>
+    <t>RHPL</t>
+  </si>
+  <si>
+    <t>3,068,670.0</t>
+  </si>
+  <si>
+    <t>SHINE</t>
+  </si>
+  <si>
+    <t>1,674,438.8</t>
+  </si>
+  <si>
+    <t>1,091,352.0</t>
+  </si>
+  <si>
+    <t>EBL</t>
+  </si>
+  <si>
+    <t>9,319,705.5</t>
+  </si>
+  <si>
+    <t>1,749,345.0</t>
+  </si>
+  <si>
+    <t>UPPER</t>
+  </si>
+  <si>
+    <t>1,055,984.8</t>
+  </si>
+  <si>
+    <t>NHPC</t>
+  </si>
+  <si>
+    <t>1,009,481.3</t>
+  </si>
+  <si>
+    <t>GVL</t>
+  </si>
+  <si>
+    <t>921,627.0</t>
+  </si>
+  <si>
+    <t>4,077,337.9</t>
+  </si>
+  <si>
+    <t>2,401,799.0</t>
+  </si>
+  <si>
+    <t>SWBBL</t>
+  </si>
+  <si>
+    <t>1,907,320.0</t>
+  </si>
+  <si>
+    <t>MEGA</t>
+  </si>
+  <si>
+    <t>1,720,255.2</t>
+  </si>
+  <si>
+    <t>961,948.1</t>
+  </si>
+  <si>
+    <t>Sell Amount</t>
+  </si>
+  <si>
+    <t>30,281,551.0</t>
+  </si>
+  <si>
+    <t>11,174,350.5</t>
+  </si>
+  <si>
+    <t>4,591,567.4</t>
+  </si>
+  <si>
+    <t>4,318,438.5</t>
+  </si>
+  <si>
+    <t>4,222,684.5</t>
+  </si>
+  <si>
+    <t>4,290,873.9</t>
+  </si>
+  <si>
+    <t>2,010,738.1</t>
+  </si>
+  <si>
+    <t>CYCL</t>
+  </si>
+  <si>
+    <t>1,578,654.8</t>
+  </si>
+  <si>
+    <t>1,054,356.0</t>
+  </si>
+  <si>
+    <t>890,580.0</t>
+  </si>
+  <si>
+    <t>4,944,722.5</t>
+  </si>
+  <si>
+    <t>CIT</t>
+  </si>
+  <si>
+    <t>4,326,112.7</t>
+  </si>
+  <si>
+    <t>3,400,516.5</t>
+  </si>
+  <si>
+    <t>SBL</t>
+  </si>
+  <si>
+    <t>2,009,037.5</t>
+  </si>
+  <si>
+    <t>NGPL</t>
+  </si>
+  <si>
+    <t>1,467,288.0</t>
+  </si>
+  <si>
+    <t>4,358,118.5</t>
+  </si>
+  <si>
+    <t>3,098,036.5</t>
+  </si>
+  <si>
+    <t>2,112,340.1</t>
+  </si>
+  <si>
+    <t>AKPL</t>
+  </si>
+  <si>
+    <t>1,550,520.0</t>
+  </si>
+  <si>
+    <t>1,033,678.8</t>
+  </si>
+  <si>
+    <t>HDHPC</t>
+  </si>
+  <si>
+    <t>4,328,188.0</t>
+  </si>
+  <si>
+    <t>4,009,086.5</t>
+  </si>
+  <si>
+    <t>GUFL</t>
+  </si>
+  <si>
+    <t>2,591,883.29</t>
+  </si>
+  <si>
+    <t>2,411,267.0</t>
+  </si>
+  <si>
+    <t>2,150,476.7</t>
+  </si>
+  <si>
+    <t>BOKL</t>
+  </si>
+  <si>
+    <t>1,148,086.7</t>
+  </si>
+  <si>
+    <t>MKJC</t>
+  </si>
+  <si>
+    <t>628,521.1</t>
   </si>
   <si>
     <t>HIDCL</t>
   </si>
   <si>
-    <t>1,004,109.0</t>
-  </si>
-  <si>
-    <t>BNT</t>
-  </si>
-  <si>
-    <t>861,000.0</t>
+    <t>613,101.5</t>
+  </si>
+  <si>
+    <t>KRBL</t>
+  </si>
+  <si>
+    <t>579,366.0</t>
+  </si>
+  <si>
+    <t>478,151.1</t>
   </si>
   <si>
     <t>NLIC</t>
   </si>
   <si>
-    <t>690,034.1</t>
-  </si>
-  <si>
-    <t>10,914,713.7</t>
-  </si>
-  <si>
-    <t>SHIVM</t>
-  </si>
-  <si>
-    <t>5,583,253.9</t>
-  </si>
-  <si>
-    <t>HDL</t>
-  </si>
-  <si>
-    <t>4,037,660.0</t>
-  </si>
-  <si>
-    <t>CCBL</t>
-  </si>
-  <si>
-    <t>3,741,567.4</t>
-  </si>
-  <si>
-    <t>NICA</t>
-  </si>
-  <si>
-    <t>3,171,268.0</t>
-  </si>
-  <si>
-    <t>11,001,634.3</t>
-  </si>
-  <si>
-    <t>5,367,052.3</t>
-  </si>
-  <si>
-    <t>3,321,009.6</t>
-  </si>
-  <si>
-    <t>SAHAS</t>
-  </si>
-  <si>
-    <t>3,153,387.0</t>
-  </si>
-  <si>
-    <t>2,861,380.5</t>
-  </si>
-  <si>
-    <t>35,700,000.0</t>
-  </si>
-  <si>
-    <t>2,344,008.0</t>
-  </si>
-  <si>
-    <t>API</t>
-  </si>
-  <si>
-    <t>1,706,972.4</t>
-  </si>
-  <si>
-    <t>UPPER</t>
-  </si>
-  <si>
-    <t>1,152,762.5</t>
-  </si>
-  <si>
-    <t>1,134,727.5</t>
-  </si>
-  <si>
-    <t>10,980,986.8</t>
-  </si>
-  <si>
-    <t>10,421,445.19</t>
-  </si>
-  <si>
-    <t>2,198,334.79</t>
-  </si>
-  <si>
-    <t>995,259.1</t>
-  </si>
-  <si>
-    <t>NMFBS</t>
-  </si>
-  <si>
-    <t>829,126.0</t>
-  </si>
-  <si>
-    <t>5,100,000.0</t>
-  </si>
-  <si>
-    <t>NMB</t>
-  </si>
-  <si>
-    <t>3,965,338.8</t>
-  </si>
-  <si>
-    <t>EBL</t>
-  </si>
-  <si>
-    <t>2,633,725.0</t>
-  </si>
-  <si>
-    <t>NTC</t>
-  </si>
-  <si>
-    <t>2,585,194.0</t>
-  </si>
-  <si>
-    <t>KSBBL</t>
-  </si>
-  <si>
-    <t>1,944,775.0</t>
-  </si>
-  <si>
-    <t>Sell Amount</t>
-  </si>
-  <si>
-    <t>18,624,520.7</t>
-  </si>
-  <si>
-    <t>14,187,045.3</t>
-  </si>
-  <si>
-    <t>13,467,368.8</t>
-  </si>
-  <si>
-    <t>10,713,099.4</t>
-  </si>
-  <si>
-    <t>3,766,193.0</t>
-  </si>
-  <si>
-    <t>930,441.0</t>
-  </si>
-  <si>
-    <t>GFCL</t>
-  </si>
-  <si>
-    <t>873,460.0</t>
-  </si>
-  <si>
-    <t>784,366.7</t>
-  </si>
-  <si>
-    <t>NHPC</t>
-  </si>
-  <si>
-    <t>752,282.4</t>
-  </si>
-  <si>
-    <t>RMDC</t>
-  </si>
-  <si>
-    <t>2,186,136.0</t>
-  </si>
-  <si>
-    <t>1,675,488.0</t>
-  </si>
-  <si>
-    <t>1,453,304.0</t>
-  </si>
-  <si>
-    <t>CYCL</t>
-  </si>
-  <si>
-    <t>1,436,305.2</t>
-  </si>
-  <si>
-    <t>1,215,673.0</t>
-  </si>
-  <si>
-    <t>UMHL</t>
-  </si>
-  <si>
-    <t>12,274,208.8</t>
+    <t>2,750,564.4</t>
+  </si>
+  <si>
+    <t>1,075,995.0</t>
+  </si>
+  <si>
+    <t>939,485.5</t>
+  </si>
+  <si>
+    <t>708,900.0</t>
   </si>
   <si>
     <t>CHCL</t>
   </si>
   <si>
-    <t>4,740,671.5</t>
-  </si>
-  <si>
-    <t>4,469,340.0</t>
-  </si>
-  <si>
-    <t>3,399,578.5</t>
-  </si>
-  <si>
-    <t>2,678,382.0</t>
-  </si>
-  <si>
-    <t>SKBBL</t>
-  </si>
-  <si>
-    <t>2,897,211.0</t>
-  </si>
-  <si>
-    <t>SSHL</t>
-  </si>
-  <si>
-    <t>1,521,070.0</t>
-  </si>
-  <si>
-    <t>987,895.0</t>
-  </si>
-  <si>
-    <t>SCB</t>
-  </si>
-  <si>
-    <t>535,593.0</t>
-  </si>
-  <si>
-    <t>HIDCLP</t>
-  </si>
-  <si>
-    <t>418,653.8</t>
-  </si>
-  <si>
-    <t>5,913,924.4</t>
-  </si>
-  <si>
-    <t>NGPL</t>
-  </si>
-  <si>
-    <t>2,654,727.9</t>
-  </si>
-  <si>
-    <t>1,748,013.4</t>
-  </si>
-  <si>
-    <t>HDHPC</t>
-  </si>
-  <si>
-    <t>690,208.0</t>
-  </si>
-  <si>
-    <t>CBBL</t>
-  </si>
-  <si>
-    <t>675,288.0</t>
-  </si>
-  <si>
-    <t>13,885,197.6</t>
-  </si>
-  <si>
-    <t>2,434,985.0</t>
-  </si>
-  <si>
-    <t>2,426,013.6</t>
-  </si>
-  <si>
-    <t>FMDBL</t>
-  </si>
-  <si>
-    <t>1,517,983.5</t>
-  </si>
-  <si>
-    <t>NLBBL</t>
-  </si>
-  <si>
-    <t>1,389,337.5</t>
+    <t>652,447.1</t>
   </si>
   <si>
     <t>Top Traded Stocks</t>
@@ -473,310 +467,322 @@
     <t>Percentage (%)</t>
   </si>
   <si>
-    <t>213,241,682.5</t>
-  </si>
-  <si>
-    <t>109,878,378.0</t>
-  </si>
-  <si>
-    <t>62,177,415.3</t>
-  </si>
-  <si>
-    <t>43,566,380.7</t>
+    <t>71,756,635.7</t>
+  </si>
+  <si>
+    <t>60,371,847.8</t>
+  </si>
+  <si>
+    <t>46,995,983.6</t>
+  </si>
+  <si>
+    <t>35,150,426.9</t>
+  </si>
+  <si>
+    <t>29,965,858.2</t>
   </si>
   <si>
     <t>Commercial Banks</t>
   </si>
   <si>
-    <t>443,539,946.8</t>
+    <t>235,380,257.2</t>
   </si>
   <si>
     <t>Hydro Power</t>
   </si>
   <si>
-    <t>231,984,841.6</t>
+    <t>152,043,362.8</t>
+  </si>
+  <si>
+    <t>Microfinance</t>
+  </si>
+  <si>
+    <t>123,339,664.6</t>
+  </si>
+  <si>
+    <t>Others</t>
+  </si>
+  <si>
+    <t>75,393,599.3</t>
+  </si>
+  <si>
+    <t>Manufacturing And Processing</t>
+  </si>
+  <si>
+    <t>60,598,512.8</t>
+  </si>
+  <si>
+    <t>Development Banks</t>
+  </si>
+  <si>
+    <t>33,519,802.1</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>28,220,599.4</t>
+  </si>
+  <si>
+    <t>Investment</t>
+  </si>
+  <si>
+    <t>20,318,537.7</t>
+  </si>
+  <si>
+    <t>Non Life Insurance</t>
+  </si>
+  <si>
+    <t>17,860,653.8</t>
+  </si>
+  <si>
+    <t>Life Insurance</t>
+  </si>
+  <si>
+    <t>16,550,785.7</t>
+  </si>
+  <si>
+    <t>Hotels And Tourism</t>
+  </si>
+  <si>
+    <t>6,278,044.0</t>
+  </si>
+  <si>
+    <t>Tradings</t>
+  </si>
+  <si>
+    <t>3,954,212.0</t>
   </si>
   <si>
     <t>Promoter Shares/debenture</t>
   </si>
   <si>
-    <t>175,487,172.0</t>
-  </si>
-  <si>
-    <t>Microfinance</t>
-  </si>
-  <si>
-    <t>150,037,867.5</t>
-  </si>
-  <si>
-    <t>Manufacturing And Processing</t>
-  </si>
-  <si>
-    <t>110,580,329.0</t>
-  </si>
-  <si>
-    <t>Development Banks</t>
-  </si>
-  <si>
-    <t>69,192,121.2</t>
-  </si>
-  <si>
-    <t>Finance</t>
-  </si>
-  <si>
-    <t>43,702,165.5</t>
-  </si>
-  <si>
-    <t>Life Insurance</t>
-  </si>
-  <si>
-    <t>37,785,185.6</t>
-  </si>
-  <si>
-    <t>Investment</t>
-  </si>
-  <si>
-    <t>34,665,877.0</t>
-  </si>
-  <si>
-    <t>Others</t>
-  </si>
-  <si>
-    <t>27,685,840.3</t>
-  </si>
-  <si>
-    <t>Non Life Insurance</t>
-  </si>
-  <si>
-    <t>26,867,295.3</t>
-  </si>
-  <si>
-    <t>Hotels And Tourism</t>
-  </si>
-  <si>
-    <t>9,301,239.6</t>
-  </si>
-  <si>
-    <t>Tradings</t>
-  </si>
-  <si>
-    <t>3,406,072.0</t>
+    <t>2,067,450.8</t>
   </si>
   <si>
     <t>Mutual Fund</t>
   </si>
   <si>
-    <t>1,774,510.62</t>
+    <t>1,563,682.95</t>
   </si>
   <si>
     <t>Total</t>
   </si>
   <si>
-    <t>10000000</t>
+    <t>777,089,165.15</t>
   </si>
   <si>
     <t>100%</t>
   </si>
   <si>
-    <t>72,151,984.1</t>
-  </si>
-  <si>
-    <t>26,614,203.7</t>
-  </si>
-  <si>
-    <t>13,666,732.3</t>
-  </si>
-  <si>
-    <t>11,932,607.4</t>
-  </si>
-  <si>
-    <t>59,477,200.0</t>
-  </si>
-  <si>
-    <t>3,719,191.7</t>
-  </si>
-  <si>
-    <t>3,406,007.4</t>
-  </si>
-  <si>
-    <t>1,958,554.0</t>
-  </si>
-  <si>
-    <t>1,898,596.8</t>
-  </si>
-  <si>
-    <t>25,894,374.8</t>
-  </si>
-  <si>
-    <t>10,876,560.6</t>
-  </si>
-  <si>
-    <t>9,620,913.9</t>
-  </si>
-  <si>
-    <t>8,489,988.4</t>
-  </si>
-  <si>
-    <t>4,675,010.9</t>
-  </si>
-  <si>
-    <t>16,217,810.5</t>
-  </si>
-  <si>
-    <t>13,962,715.7</t>
-  </si>
-  <si>
-    <t>8,688,061.9</t>
-  </si>
-  <si>
-    <t>8,442,086.0</t>
-  </si>
-  <si>
-    <t>3,258,094.5</t>
-  </si>
-  <si>
-    <t>35,897,475.0</t>
-  </si>
-  <si>
-    <t>6,628,452.4</t>
-  </si>
-  <si>
-    <t>3,543,787.7</t>
-  </si>
-  <si>
-    <t>3,016,469.3</t>
-  </si>
-  <si>
-    <t>3,006,786.0</t>
-  </si>
-  <si>
-    <t>23,764,310.4</t>
-  </si>
-  <si>
-    <t>4,492,383.2</t>
-  </si>
-  <si>
-    <t>4,434,140.4</t>
-  </si>
-  <si>
-    <t>2,935,734.8</t>
-  </si>
-  <si>
-    <t>1,647,569.5</t>
-  </si>
-  <si>
-    <t>12,210,602.6</t>
-  </si>
-  <si>
-    <t>4,273,194.8</t>
-  </si>
-  <si>
-    <t>4,192,627.8</t>
-  </si>
-  <si>
-    <t>3,994,035.0</t>
-  </si>
-  <si>
-    <t>59,952,500.0</t>
-  </si>
-  <si>
-    <t>58,006,145.1</t>
-  </si>
-  <si>
-    <t>29,059,169.0</t>
-  </si>
-  <si>
-    <t>10,496,575.5</t>
-  </si>
-  <si>
-    <t>7,313,307.4</t>
-  </si>
-  <si>
-    <t>7,343,225.2</t>
-  </si>
-  <si>
-    <t>3,307,998.2</t>
-  </si>
-  <si>
-    <t>1,986,986.6</t>
-  </si>
-  <si>
-    <t>1,852,409.4</t>
-  </si>
-  <si>
-    <t>7,412,950.9</t>
-  </si>
-  <si>
-    <t>6,547,137.6</t>
-  </si>
-  <si>
-    <t>5,164,426.09</t>
-  </si>
-  <si>
-    <t>3,256,072.0</t>
-  </si>
-  <si>
-    <t>1,509,576.0</t>
-  </si>
-  <si>
-    <t>25,781,444.6</t>
-  </si>
-  <si>
-    <t>9,018,665.19</t>
-  </si>
-  <si>
-    <t>8,327,418.7</t>
-  </si>
-  <si>
-    <t>5,605,274.8</t>
-  </si>
-  <si>
-    <t>5,590,603.0</t>
-  </si>
-  <si>
-    <t>4,284,650.2</t>
-  </si>
-  <si>
-    <t>3,075,956.5</t>
-  </si>
-  <si>
-    <t>3,021,438.0</t>
-  </si>
-  <si>
-    <t>916,874.4</t>
-  </si>
-  <si>
-    <t>768,173.0</t>
-  </si>
-  <si>
-    <t>9,918,070.8</t>
-  </si>
-  <si>
-    <t>6,485,669.0</t>
-  </si>
-  <si>
-    <t>2,645,069.0</t>
-  </si>
-  <si>
-    <t>1,397,438.8</t>
-  </si>
-  <si>
-    <t>1,108,835.0</t>
-  </si>
-  <si>
-    <t>17,533,706.39</t>
-  </si>
-  <si>
-    <t>11,695,745.9</t>
-  </si>
-  <si>
-    <t>4,232,313.8</t>
-  </si>
-  <si>
-    <t>1,459,430.0</t>
-  </si>
-  <si>
-    <t>1,085,445.3</t>
+    <t>48,853,869.4</t>
+  </si>
+  <si>
+    <t>21,836,671.9</t>
+  </si>
+  <si>
+    <t>12,080,788.8</t>
+  </si>
+  <si>
+    <t>5,774,600.8</t>
+  </si>
+  <si>
+    <t>2,599,600.1</t>
+  </si>
+  <si>
+    <t>18,151,654.5</t>
+  </si>
+  <si>
+    <t>11,698,428.1</t>
+  </si>
+  <si>
+    <t>9,179,562.5</t>
+  </si>
+  <si>
+    <t>5,449,554.9</t>
+  </si>
+  <si>
+    <t>3,316,500.1</t>
+  </si>
+  <si>
+    <t>10,977,290.7</t>
+  </si>
+  <si>
+    <t>10,442,923.6</t>
+  </si>
+  <si>
+    <t>5,723,983.0</t>
+  </si>
+  <si>
+    <t>4,662,824.0</t>
+  </si>
+  <si>
+    <t>4,370,917.4</t>
+  </si>
+  <si>
+    <t>7,123,390.1</t>
+  </si>
+  <si>
+    <t>5,290,166.4</t>
+  </si>
+  <si>
+    <t>3,733,438.1</t>
+  </si>
+  <si>
+    <t>3,116,418.0</t>
+  </si>
+  <si>
+    <t>2,701,235.7</t>
+  </si>
+  <si>
+    <t>8,886,870.6</t>
+  </si>
+  <si>
+    <t>6,411,027.0</t>
+  </si>
+  <si>
+    <t>3,953,552.4</t>
+  </si>
+  <si>
+    <t>1,616,365.5</t>
+  </si>
+  <si>
+    <t>1,315,962.39</t>
+  </si>
+  <si>
+    <t>12,306,543.4</t>
+  </si>
+  <si>
+    <t>3,929,686.1</t>
+  </si>
+  <si>
+    <t>1,378,050.0</t>
+  </si>
+  <si>
+    <t>943,444.0</t>
+  </si>
+  <si>
+    <t>808,415.0</t>
+  </si>
+  <si>
+    <t>8,531,078.69</t>
+  </si>
+  <si>
+    <t>3,475,748.4</t>
+  </si>
+  <si>
+    <t>3,227,697.9</t>
+  </si>
+  <si>
+    <t>2,415,799.0</t>
+  </si>
+  <si>
+    <t>1,061,079.0</t>
+  </si>
+  <si>
+    <t>48,181,674.7</t>
+  </si>
+  <si>
+    <t>9,091,611.6</t>
+  </si>
+  <si>
+    <t>8,541,123.0</t>
+  </si>
+  <si>
+    <t>5,102,469.9</t>
+  </si>
+  <si>
+    <t>3,056,254.8</t>
+  </si>
+  <si>
+    <t>5,719,173.6</t>
+  </si>
+  <si>
+    <t>5,293,286.3</t>
+  </si>
+  <si>
+    <t>5,018,215.9</t>
+  </si>
+  <si>
+    <t>4,904,360.9</t>
+  </si>
+  <si>
+    <t>1,371,519.4</t>
+  </si>
+  <si>
+    <t>10,816,521.7</t>
+  </si>
+  <si>
+    <t>8,396,955.69</t>
+  </si>
+  <si>
+    <t>5,359,906.5</t>
+  </si>
+  <si>
+    <t>4,570,611.59</t>
+  </si>
+  <si>
+    <t>4,141,591.6</t>
+  </si>
+  <si>
+    <t>6,824,340.4</t>
+  </si>
+  <si>
+    <t>6,126,170.5</t>
+  </si>
+  <si>
+    <t>4,510,063.3</t>
+  </si>
+  <si>
+    <t>1,936,280.0</t>
+  </si>
+  <si>
+    <t>1,073,174.7</t>
+  </si>
+  <si>
+    <t>10,469,477.1</t>
+  </si>
+  <si>
+    <t>2,787,055.9</t>
+  </si>
+  <si>
+    <t>2,783,817.0</t>
+  </si>
+  <si>
+    <t>2,651,405.7</t>
+  </si>
+  <si>
+    <t>2,600,467.2</t>
+  </si>
+  <si>
+    <t>3,442,376.4</t>
+  </si>
+  <si>
+    <t>1,994,863.7</t>
+  </si>
+  <si>
+    <t>915,814.3</t>
+  </si>
+  <si>
+    <t>860,027.6</t>
+  </si>
+  <si>
+    <t>642,246.0</t>
+  </si>
+  <si>
+    <t>3,949,391.5</t>
+  </si>
+  <si>
+    <t>3,484,865.1</t>
+  </si>
+  <si>
+    <t>2,997,350.9</t>
+  </si>
+  <si>
+    <t>1,705,876.9</t>
+  </si>
+  <si>
+    <t>1,564,014.0</t>
   </si>
 </sst>
 </file>
@@ -1403,7 +1409,7 @@
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
       <c r="T4" s="6" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U4" s="6"/>
       <c r="V4" s="6"/>
@@ -1413,37 +1419,37 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R5" s="5"/>
       <c r="S5" s="5"/>
       <c r="T5" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="U5" s="6"/>
       <c r="V5" s="6"/>
@@ -1453,37 +1459,37 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
       <c r="N6" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
       <c r="Q6" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R6" s="7"/>
       <c r="S6" s="7"/>
       <c r="T6" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="U6" s="7"/>
       <c r="V6" s="7"/>
@@ -1493,296 +1499,296 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
       <c r="E7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
       <c r="K7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
       <c r="N7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
       <c r="Q7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="R7" s="8"/>
       <c r="S7" s="8"/>
       <c r="T7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="U7" s="8"/>
       <c r="V7" s="8"/>
     </row>
     <row r="8" spans="1:22">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="E8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="H8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="J8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="K8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="M8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M8" s="5" t="s">
-        <v>40</v>
-      </c>
       <c r="N8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="O8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="O8" s="6" t="s">
+      <c r="P8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="P8" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="Q8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="R8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R8" s="5" t="s">
+      <c r="S8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="S8" s="5" t="s">
-        <v>40</v>
-      </c>
       <c r="T8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="U8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="U8" s="6" t="s">
+      <c r="V8" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="V8" s="6" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:22">
       <c r="A9" s="1"/>
       <c r="B9" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>42</v>
-      </c>
       <c r="D9" s="10">
-        <v>0.264227647636373</v>
+        <v>0.3126015836481585</v>
       </c>
       <c r="E9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="11" t="s">
-        <v>52</v>
-      </c>
       <c r="G9" s="12">
-        <v>0.790368628354411</v>
+        <v>0.1833618595784118</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J9" s="14">
-        <v>0.1655933372948122</v>
+        <v>0.1503102929396203</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="L9" s="15" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="M9" s="16">
-        <v>0.1877339767060771</v>
+        <v>0.1428459490624485</v>
       </c>
       <c r="N9" s="17" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="O9" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="P9" s="18">
-        <v>0.6491619096994145</v>
+        <v>0.1532691878548762</v>
       </c>
       <c r="Q9" s="15" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="R9" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S9" s="16">
-        <v>0.262234259014455</v>
+        <v>0.4285672780907033</v>
       </c>
       <c r="T9" s="17" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="U9" s="17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="V9" s="18">
-        <v>0.1272107770755374</v>
+        <v>0.1902378102627345</v>
       </c>
     </row>
     <row r="10" spans="1:22">
       <c r="A10" s="1"/>
       <c r="B10" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>44</v>
-      </c>
       <c r="D10" s="10">
-        <v>0.0746852926835172</v>
+        <v>0.1419179650747541</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G10" s="12">
-        <v>0.03297939281130662</v>
+        <v>0.1222815773313923</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="I10" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="J10" s="14">
+        <v>0.09020809453489893</v>
+      </c>
+      <c r="K10" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="L10" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="M10" s="16">
+        <v>0.1056010283350162</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="O10" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="P10" s="18">
+        <v>0.121493998693807</v>
+      </c>
+      <c r="Q10" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="J10" s="14">
-        <v>0.08470672448928053</v>
-      </c>
-      <c r="K10" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="L10" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="M10" s="16">
-        <v>0.09158439955311889</v>
-      </c>
-      <c r="N10" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="O10" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="P10" s="18">
-        <v>0.04262298906528586</v>
-      </c>
-      <c r="Q10" s="15" t="s">
-        <v>67</v>
-      </c>
       <c r="R10" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="S10" s="16">
-        <v>0.2488719829698501</v>
+        <v>0.08044374632777627</v>
       </c>
       <c r="T10" s="17" t="s">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="U10" s="17" t="s">
         <v>90</v>
       </c>
       <c r="V10" s="18">
-        <v>0.09890859414034885</v>
+        <v>0.11206159353416</v>
       </c>
     </row>
     <row r="11" spans="1:22">
       <c r="A11" s="1"/>
       <c r="B11" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>46</v>
-      </c>
       <c r="D11" s="10">
-        <v>0.07332431616937976</v>
+        <v>0.1075095996835127</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G11" s="12">
-        <v>0.01337179870342577</v>
+        <v>0.09946095761336185</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="J11" s="14">
-        <v>0.06125763924176696</v>
+        <v>0.07922009486025627</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="L11" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M11" s="16">
-        <v>0.05667033841390805</v>
+        <v>0.05754201983085062</v>
       </c>
       <c r="N11" s="17" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="O11" s="17" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="P11" s="18">
-        <v>0.03103925666633593</v>
+        <v>0.1213195075369003</v>
       </c>
       <c r="Q11" s="15" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="R11" s="15" t="s">
         <v>84</v>
       </c>
       <c r="S11" s="16">
-        <v>0.05249789548455609</v>
+        <v>0.04855953135441412</v>
       </c>
       <c r="T11" s="17" t="s">
         <v>91</v>
@@ -1791,64 +1797,64 @@
         <v>92</v>
       </c>
       <c r="V11" s="18">
-        <v>0.06569376546142545</v>
+        <v>0.08899051027149818</v>
       </c>
     </row>
     <row r="12" spans="1:22">
       <c r="A12" s="1"/>
       <c r="B12" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>48</v>
-      </c>
       <c r="D12" s="10">
-        <v>0.06610032502969335</v>
+        <v>0.08289097207907314</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G12" s="12">
-        <v>0.01146600486964023</v>
+        <v>0.09009980075765503</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J12" s="14">
-        <v>0.0567654497872421</v>
+        <v>0.06290346282550319</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L12" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="M12" s="16">
-        <v>0.05380999453901557</v>
+        <v>0.03793602279724068</v>
       </c>
       <c r="N12" s="17" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="O12" s="17" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="P12" s="18">
-        <v>0.02096161081036054</v>
+        <v>0.06619874102353082</v>
       </c>
       <c r="Q12" s="15" t="s">
-        <v>58</v>
+        <v>85</v>
       </c>
       <c r="R12" s="15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="S12" s="16">
-        <v>0.02376753905358427</v>
+        <v>0.04642106480987674</v>
       </c>
       <c r="T12" s="17" t="s">
         <v>93</v>
@@ -1857,285 +1863,285 @@
         <v>94</v>
       </c>
       <c r="V12" s="18">
-        <v>0.06448324267274841</v>
+        <v>0.08026256110416613</v>
       </c>
     </row>
     <row r="13" spans="1:22">
       <c r="A13" s="1"/>
       <c r="B13" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>50</v>
-      </c>
       <c r="D13" s="10">
-        <v>0.0507550355027225</v>
+        <v>0.04945092419600405</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G13" s="12">
-        <v>0.009189238502692005</v>
+        <v>0.05358352617353043</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="J13" s="14">
-        <v>0.04811311281359991</v>
+        <v>0.0563853125831705</v>
       </c>
       <c r="K13" s="15" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="L13" s="15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="M13" s="16">
-        <v>0.04882714017627574</v>
+        <v>0.03678756170121861</v>
       </c>
       <c r="N13" s="17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O13" s="17" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="P13" s="18">
-        <v>0.02063366585121687</v>
+        <v>0.04314647296366544</v>
       </c>
       <c r="Q13" s="15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="R13" s="15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="S13" s="16">
-        <v>0.01980015514084936</v>
+        <v>0.04238107897346119</v>
       </c>
       <c r="T13" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="U13" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="U13" s="17" t="s">
-        <v>96</v>
-      </c>
       <c r="V13" s="18">
-        <v>0.0485090860758977</v>
+        <v>0.04488195597681467</v>
       </c>
     </row>
     <row r="15" spans="1:22">
       <c r="A15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="C15" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P15" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R15" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="S15" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="V15" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:22">
       <c r="A16" s="1"/>
       <c r="B16" s="9" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>52</v>
+        <v>97</v>
       </c>
       <c r="D16" s="10">
-        <v>0.3074884487689949</v>
+        <v>0.3117491221580984</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="F16" s="11" t="s">
         <v>102</v>
       </c>
       <c r="G16" s="12">
-        <v>0.05015468905691633</v>
+        <v>0.08425293288395362</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>109</v>
+        <v>42</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J16" s="14">
-        <v>0.03316711422493213</v>
+        <v>0.1147144800624243</v>
       </c>
       <c r="K16" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="L16" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="L16" s="15" t="s">
-        <v>117</v>
-      </c>
       <c r="M16" s="16">
-        <v>0.2094494296129009</v>
+        <v>0.1521894199651549</v>
       </c>
       <c r="N16" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="O16" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="O16" s="17" t="s">
-        <v>124</v>
-      </c>
       <c r="P16" s="18">
-        <v>0.05268232564599861</v>
+        <v>0.1711144035321887</v>
       </c>
       <c r="Q16" s="15" t="s">
-        <v>43</v>
+        <v>129</v>
       </c>
       <c r="R16" s="15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="S16" s="16">
-        <v>0.1412289816158877</v>
+        <v>0.05279484335971108</v>
       </c>
       <c r="T16" s="17" t="s">
-        <v>43</v>
+        <v>138</v>
       </c>
       <c r="U16" s="17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="V16" s="18">
-        <v>0.3463425052045858</v>
+        <v>0.128334065332832</v>
       </c>
     </row>
     <row r="17" spans="1:22">
       <c r="A17" s="1"/>
       <c r="B17" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>98</v>
       </c>
       <c r="D17" s="10">
-        <v>0.0964924175081556</v>
+        <v>0.115040143058125</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F17" s="11" t="s">
         <v>103</v>
       </c>
       <c r="G17" s="12">
-        <v>0.01239075614043313</v>
+        <v>0.03948160354619333</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>61</v>
+        <v>109</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J17" s="14">
-        <v>0.02541978261119303</v>
+        <v>0.1003631182684065</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>118</v>
+        <v>62</v>
       </c>
       <c r="L17" s="15" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="M17" s="16">
-        <v>0.08089571864356222</v>
+        <v>0.1081862225558756</v>
       </c>
       <c r="N17" s="17" t="s">
-        <v>125</v>
+        <v>54</v>
       </c>
       <c r="O17" s="17" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="P17" s="18">
-        <v>0.02765884330494365</v>
+        <v>0.1584987632599254</v>
       </c>
       <c r="Q17" s="15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="R17" s="15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="S17" s="16">
-        <v>0.06339690743836429</v>
+        <v>0.02890258464171156</v>
       </c>
       <c r="T17" s="17" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="U17" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="V17" s="18">
-        <v>0.06073653608181912</v>
+        <v>0.05020308291192913</v>
       </c>
     </row>
     <row r="18" spans="1:22">
       <c r="A18" s="1"/>
       <c r="B18" s="9" t="s">
-        <v>45</v>
+        <v>83</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>99</v>
       </c>
       <c r="D18" s="10">
-        <v>0.07350214914764043</v>
+        <v>0.04727027047854128</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>104</v>
@@ -2144,408 +2150,408 @@
         <v>105</v>
       </c>
       <c r="G18" s="12">
-        <v>0.01163193567181877</v>
+        <v>0.03099748443116243</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J18" s="14">
-        <v>0.02204890261701502</v>
+        <v>0.07888986333230934</v>
       </c>
       <c r="K18" s="15" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="L18" s="15" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="M18" s="16">
-        <v>0.07626566640663003</v>
+        <v>0.07376481722287666</v>
       </c>
       <c r="N18" s="17" t="s">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="O18" s="17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P18" s="18">
-        <v>0.01796369201071437</v>
+        <v>0.1024698014283439</v>
       </c>
       <c r="Q18" s="15" t="s">
-        <v>67</v>
+        <v>133</v>
       </c>
       <c r="R18" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="S18" s="16">
-        <v>0.04174388031286388</v>
+        <v>0.02819351330879794</v>
       </c>
       <c r="T18" s="17" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="U18" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="V18" s="18">
-        <v>0.06051275985329844</v>
+        <v>0.04383391042807373</v>
       </c>
     </row>
     <row r="19" spans="1:22">
       <c r="A19" s="1"/>
       <c r="B19" s="9" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>100</v>
       </c>
       <c r="D19" s="10">
-        <v>0.06977355250736243</v>
+        <v>0.04445840345062692</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>106</v>
       </c>
       <c r="G19" s="12">
-        <v>0.0104454731728033</v>
+        <v>0.02070267907518648</v>
       </c>
       <c r="H19" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="I19" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="I19" s="13" t="s">
-        <v>114</v>
-      </c>
       <c r="J19" s="14">
-        <v>0.02179100414167462</v>
+        <v>0.04660841781078975</v>
       </c>
       <c r="K19" s="15" t="s">
-        <v>67</v>
+        <v>119</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M19" s="16">
-        <v>0.05801105304231759</v>
+        <v>0.05414555373938823</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>128</v>
+        <v>77</v>
       </c>
       <c r="O19" s="17" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="P19" s="18">
-        <v>0.009739119739541694</v>
+        <v>0.09532915725052842</v>
       </c>
       <c r="Q19" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="R19" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="R19" s="15" t="s">
-        <v>137</v>
-      </c>
       <c r="S19" s="16">
-        <v>0.01648268837240101</v>
+        <v>0.02664218409458308</v>
       </c>
       <c r="T19" s="17" t="s">
-        <v>143</v>
+        <v>50</v>
       </c>
       <c r="U19" s="17" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="V19" s="18">
-        <v>0.0378635020829106</v>
+        <v>0.03307540042125341</v>
       </c>
     </row>
     <row r="20" spans="1:22">
       <c r="A20" s="1"/>
       <c r="B20" s="9" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>101</v>
       </c>
       <c r="D20" s="10">
-        <v>0.05550386379130665</v>
+        <v>0.04347261426687188</v>
       </c>
       <c r="E20" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="F20" s="11" t="s">
-        <v>108</v>
-      </c>
       <c r="G20" s="12">
-        <v>0.01001820402060934</v>
+        <v>0.01748687533506669</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>43</v>
+        <v>114</v>
       </c>
       <c r="I20" s="13" t="s">
         <v>115</v>
       </c>
       <c r="J20" s="14">
-        <v>0.0184436673890215</v>
+        <v>0.03404016707142504</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L20" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M20" s="16">
-        <v>0.04570441902417863</v>
+        <v>0.03609699392117893</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>130</v>
+        <v>46</v>
       </c>
       <c r="O20" s="17" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="P20" s="18">
-        <v>0.007612719896664334</v>
+        <v>0.08501884341215529</v>
       </c>
       <c r="Q20" s="15" t="s">
-        <v>138</v>
+        <v>112</v>
       </c>
       <c r="R20" s="15" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="S20" s="16">
-        <v>0.01612638750292945</v>
+        <v>0.02198781017737907</v>
       </c>
       <c r="T20" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="U20" s="17" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="V20" s="18">
-        <v>0.0346546476461146</v>
+        <v>0.0304414573087679</v>
       </c>
     </row>
     <row r="23" spans="1:22">
       <c r="B23" s="19" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:22">
       <c r="B24" s="20" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="25" spans="1:22">
       <c r="B25" s="20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26" spans="1:22">
       <c r="B26" s="20" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="27" spans="1:22">
       <c r="B27" s="20" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>52</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" spans="1:22">
       <c r="B28" s="20" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="30" spans="1:22">
       <c r="B30" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="D30" s="19" t="s">
         <v>149</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="D30" s="19" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="31" spans="1:22">
       <c r="B31" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="C31" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="C31" s="21" t="s">
-        <v>157</v>
-      </c>
       <c r="D31" s="22">
-        <v>44.35399468</v>
+        <v>0.3028999344683502</v>
       </c>
     </row>
     <row r="32" spans="1:22">
       <c r="B32" s="20" t="s">
+        <v>157</v>
+      </c>
+      <c r="C32" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="C32" s="21" t="s">
-        <v>159</v>
-      </c>
       <c r="D32" s="22">
-        <v>23.19848416</v>
+        <v>0.1956575507916796</v>
       </c>
     </row>
     <row r="33" spans="2:4">
       <c r="B33" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="C33" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="C33" s="21" t="s">
-        <v>161</v>
-      </c>
       <c r="D33" s="22">
-        <v>17.5487172</v>
+        <v>0.1587200930490286</v>
       </c>
     </row>
     <row r="34" spans="2:4">
       <c r="B34" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="C34" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="C34" s="21" t="s">
-        <v>163</v>
-      </c>
       <c r="D34" s="22">
-        <v>15.00378675</v>
+        <v>0.09702052567602962</v>
       </c>
     </row>
     <row r="35" spans="2:4">
       <c r="B35" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="C35" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="C35" s="21" t="s">
-        <v>165</v>
-      </c>
       <c r="D35" s="22">
-        <v>11.0580329</v>
+        <v>0.07798141515498133</v>
       </c>
     </row>
     <row r="36" spans="2:4">
       <c r="B36" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="C36" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="C36" s="21" t="s">
-        <v>167</v>
-      </c>
       <c r="D36" s="22">
-        <v>6.91921212</v>
+        <v>0.04313507844821095</v>
       </c>
     </row>
     <row r="37" spans="2:4">
       <c r="B37" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="C37" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="C37" s="21" t="s">
-        <v>169</v>
-      </c>
       <c r="D37" s="22">
-        <v>4.37021655</v>
+        <v>0.03631578030630839</v>
       </c>
     </row>
     <row r="38" spans="2:4">
       <c r="B38" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="C38" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="C38" s="21" t="s">
-        <v>171</v>
-      </c>
       <c r="D38" s="22">
-        <v>3.77851856</v>
+        <v>0.02614698365544442</v>
       </c>
     </row>
     <row r="39" spans="2:4">
       <c r="B39" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="C39" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="C39" s="21" t="s">
-        <v>173</v>
-      </c>
       <c r="D39" s="22">
-        <v>3.4665877</v>
+        <v>0.02298404687775102</v>
       </c>
     </row>
     <row r="40" spans="2:4">
       <c r="B40" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="C40" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="C40" s="21" t="s">
-        <v>175</v>
-      </c>
       <c r="D40" s="22">
-        <v>2.76858403</v>
+        <v>0.02129843838036943</v>
       </c>
     </row>
     <row r="41" spans="2:4">
       <c r="B41" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="C41" s="21" t="s">
         <v>176</v>
       </c>
-      <c r="C41" s="21" t="s">
-        <v>177</v>
-      </c>
       <c r="D41" s="22">
-        <v>2.68672953</v>
+        <v>0.008078923605617589</v>
       </c>
     </row>
     <row r="42" spans="2:4">
       <c r="B42" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="C42" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="C42" s="21" t="s">
-        <v>179</v>
-      </c>
       <c r="D42" s="22">
-        <v>0.93012396</v>
+        <v>0.005088491999803814</v>
       </c>
     </row>
     <row r="43" spans="2:4">
       <c r="B43" s="20" t="s">
+        <v>179</v>
+      </c>
+      <c r="C43" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="C43" s="21" t="s">
-        <v>181</v>
-      </c>
       <c r="D43" s="22">
-        <v>0.3406072</v>
+        <v>0.002660506532221337</v>
       </c>
     </row>
     <row r="44" spans="2:4">
       <c r="B44" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="C44" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="C44" s="21" t="s">
-        <v>183</v>
-      </c>
       <c r="D44" s="22">
-        <v>0.177451062</v>
+        <v>0.002012231054203626</v>
       </c>
     </row>
     <row r="45" spans="2:4">
       <c r="B45" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C45" s="20" t="s">
         <v>184</v>
       </c>
-      <c r="C45" s="20" t="s">
+      <c r="D45" s="20" t="s">
         <v>185</v>
-      </c>
-      <c r="D45" s="20" t="s">
-        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2728,7 +2734,7 @@
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
       <c r="T4" s="6" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="U4" s="6"/>
       <c r="V4" s="6"/>
@@ -2738,37 +2744,37 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R5" s="5"/>
       <c r="S5" s="5"/>
       <c r="T5" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="U5" s="6"/>
       <c r="V5" s="6"/>
@@ -2778,37 +2784,37 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
       <c r="N6" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
       <c r="Q6" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R6" s="7"/>
       <c r="S6" s="7"/>
       <c r="T6" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="U6" s="7"/>
       <c r="V6" s="7"/>
@@ -2818,835 +2824,835 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
       <c r="E7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
       <c r="K7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
       <c r="N7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
       <c r="Q7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="R7" s="8"/>
       <c r="S7" s="8"/>
       <c r="T7" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="U7" s="8"/>
       <c r="V7" s="8"/>
     </row>
     <row r="8" spans="1:22">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="E8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="H8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="J8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="K8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="M8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M8" s="5" t="s">
-        <v>40</v>
-      </c>
       <c r="N8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="O8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="O8" s="6" t="s">
+      <c r="P8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="P8" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="Q8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="R8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R8" s="5" t="s">
+      <c r="S8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="S8" s="5" t="s">
-        <v>40</v>
-      </c>
       <c r="T8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="U8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="U8" s="6" t="s">
+      <c r="V8" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="V8" s="6" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:22">
       <c r="A9" s="1"/>
       <c r="B9" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D9" s="10">
-        <v>0.3738146868831371</v>
+        <v>0.5029514802420914</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F9" s="11" t="s">
         <v>191</v>
       </c>
       <c r="G9" s="12">
-        <v>0.7920625607811453</v>
+        <v>0.3564146055005752</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I9" s="13" t="s">
         <v>196</v>
       </c>
       <c r="J9" s="14">
-        <v>0.3928583065165223</v>
+        <v>0.2546663023343749</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L9" s="15" t="s">
         <v>201</v>
       </c>
       <c r="M9" s="16">
-        <v>0.2767437978401602</v>
+        <v>0.2487551927522225</v>
       </c>
       <c r="N9" s="17" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="O9" s="17" t="s">
         <v>206</v>
       </c>
       <c r="P9" s="18">
-        <v>0.65275275698563</v>
+        <v>0.3513413839663952</v>
       </c>
       <c r="Q9" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R9" s="15" t="s">
         <v>211</v>
       </c>
       <c r="S9" s="16">
-        <v>0.5675096821656781</v>
+        <v>0.5659172178394596</v>
       </c>
       <c r="T9" s="17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="U9" s="17" t="s">
         <v>216</v>
       </c>
       <c r="V9" s="18">
-        <v>0.3045725971189368</v>
+        <v>0.3980375850299421</v>
       </c>
     </row>
     <row r="10" spans="1:22">
       <c r="A10" s="1"/>
       <c r="B10" s="9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>42</v>
+        <v>187</v>
       </c>
       <c r="D10" s="10">
-        <v>0.264227647636373</v>
+        <v>0.2248089371538272</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F10" s="11" t="s">
         <v>192</v>
       </c>
       <c r="G10" s="12">
-        <v>0.04952876903986706</v>
+        <v>0.2297030629487986</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I10" s="13" t="s">
         <v>197</v>
       </c>
       <c r="J10" s="14">
-        <v>0.1650144948871416</v>
+        <v>0.2422693186737214</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L10" s="15" t="s">
         <v>202</v>
       </c>
       <c r="M10" s="16">
-        <v>0.238262431971346</v>
+        <v>0.1847373713989539</v>
       </c>
       <c r="N10" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O10" s="17" t="s">
         <v>207</v>
       </c>
       <c r="P10" s="18">
-        <v>0.1205304991130439</v>
+        <v>0.2534591984298643</v>
       </c>
       <c r="Q10" s="15" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="R10" s="15" t="s">
         <v>212</v>
       </c>
       <c r="S10" s="16">
-        <v>0.1072815040321318</v>
+        <v>0.1807068770175057</v>
       </c>
       <c r="T10" s="17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="U10" s="17" t="s">
-        <v>88</v>
+        <v>217</v>
       </c>
       <c r="V10" s="18">
-        <v>0.1272107770755374</v>
+        <v>0.1621692341564831</v>
       </c>
     </row>
     <row r="11" spans="1:22">
       <c r="A11" s="1"/>
       <c r="B11" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>188</v>
       </c>
       <c r="D11" s="10">
-        <v>0.1378864399483579</v>
+        <v>0.1243719419582368</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F11" s="11" t="s">
         <v>193</v>
       </c>
       <c r="G11" s="12">
-        <v>0.0453580690295362</v>
+        <v>0.1802441836420682</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="I11" s="13" t="s">
         <v>198</v>
       </c>
       <c r="J11" s="14">
-        <v>0.1459643637310475</v>
+        <v>0.1327928379663683</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="L11" s="15" t="s">
         <v>203</v>
       </c>
       <c r="M11" s="16">
-        <v>0.148254737967027</v>
+        <v>0.1303750182366106</v>
       </c>
       <c r="N11" s="17" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="O11" s="17" t="s">
         <v>208</v>
       </c>
       <c r="P11" s="18">
-        <v>0.06443955156586263</v>
+        <v>0.1563032291479144</v>
       </c>
       <c r="Q11" s="15" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="R11" s="15" t="s">
         <v>213</v>
       </c>
       <c r="S11" s="16">
-        <v>0.1058906219758009</v>
+        <v>0.06336972102529352</v>
       </c>
       <c r="T11" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="U11" s="17" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="V11" s="18">
-        <v>0.1065875355104207</v>
+        <v>0.1505958534085749</v>
       </c>
     </row>
     <row r="12" spans="1:22">
       <c r="A12" s="1"/>
       <c r="B12" s="9" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>189</v>
       </c>
       <c r="D12" s="10">
-        <v>0.07080644169617722</v>
+        <v>0.05944962099905161</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F12" s="11" t="s">
         <v>194</v>
       </c>
       <c r="G12" s="12">
-        <v>0.02608221800401087</v>
+        <v>0.1070040728153583</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I12" s="13" t="s">
         <v>199</v>
       </c>
       <c r="J12" s="14">
-        <v>0.1288064489268503</v>
+        <v>0.1081746105636047</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="L12" s="15" t="s">
         <v>204</v>
       </c>
       <c r="M12" s="16">
-        <v>0.1440573585030634</v>
+        <v>0.1088281210777009</v>
       </c>
       <c r="N12" s="17" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="O12" s="17" t="s">
         <v>209</v>
       </c>
       <c r="P12" s="18">
-        <v>0.05485089555567663</v>
+        <v>0.06390281993816073</v>
       </c>
       <c r="Q12" s="15" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="R12" s="15" t="s">
         <v>214</v>
       </c>
       <c r="S12" s="16">
-        <v>0.07010756446232584</v>
+        <v>0.04338433517142849</v>
       </c>
       <c r="T12" s="17" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="U12" s="17" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="V12" s="18">
-        <v>0.1045779294953923</v>
+        <v>0.112714796533028</v>
       </c>
     </row>
     <row r="13" spans="1:22">
       <c r="A13" s="1"/>
       <c r="B13" s="9" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>190</v>
       </c>
       <c r="D13" s="10">
-        <v>0.06182205457785054</v>
+        <v>0.02676293064173314</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F13" s="11" t="s">
         <v>195</v>
       </c>
       <c r="G13" s="12">
-        <v>0.02528376324539299</v>
+        <v>0.06512073457458757</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="I13" s="13" t="s">
         <v>200</v>
       </c>
       <c r="J13" s="14">
-        <v>0.07092725270664897</v>
+        <v>0.1014025593826152</v>
       </c>
       <c r="K13" s="15" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="L13" s="15" t="s">
         <v>205</v>
       </c>
       <c r="M13" s="16">
-        <v>0.05559674320107131</v>
+        <v>0.09432958153206925</v>
       </c>
       <c r="N13" s="17" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="O13" s="17" t="s">
         <v>210</v>
       </c>
       <c r="P13" s="18">
-        <v>0.05467481629740795</v>
+        <v>0.05202641871073704</v>
       </c>
       <c r="Q13" s="15" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="R13" s="15" t="s">
         <v>215</v>
       </c>
       <c r="S13" s="16">
-        <v>0.03934520411292327</v>
+        <v>0.03717501761377502</v>
       </c>
       <c r="T13" s="17" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="U13" s="17" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="V13" s="18">
-        <v>0.09962437176801846</v>
+        <v>0.04950714177399231</v>
       </c>
     </row>
     <row r="15" spans="1:22">
       <c r="A15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="C15" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P15" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R15" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="S15" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="V15" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:22">
       <c r="A16" s="1"/>
       <c r="B16" s="9" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D16" s="10">
-        <v>0.3106099616650912</v>
+        <v>0.4960312234942014</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G16" s="12">
-        <v>0.09779030882934364</v>
+        <v>0.1122981380255615</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="J16" s="14">
-        <v>0.1124660996589935</v>
+        <v>0.2509365617381825</v>
       </c>
       <c r="K16" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L16" s="15" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="M16" s="16">
-        <v>0.4399394660832725</v>
+        <v>0.238312108108298</v>
       </c>
       <c r="N16" s="17" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="O16" s="17" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="P16" s="18">
-        <v>0.07791125227523749</v>
+        <v>0.4139095458100269</v>
       </c>
       <c r="Q16" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="R16" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="S16" s="16">
-        <v>0.2368510220858205</v>
+        <v>0.1582979080091827</v>
       </c>
       <c r="T16" s="17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="U16" s="17" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="V16" s="18">
-        <v>0.437348316893789</v>
+        <v>0.1842681693931368</v>
       </c>
     </row>
     <row r="17" spans="1:22">
       <c r="A17" s="1"/>
       <c r="B17" s="9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D17" s="10">
-        <v>0.3005260248671985</v>
+        <v>0.09359830793681552</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G17" s="12">
-        <v>0.0440528727874113</v>
+        <v>0.1039356797153725</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="J17" s="14">
-        <v>0.0993303530180867</v>
+        <v>0.1948041386008437</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="L17" s="15" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="M17" s="16">
-        <v>0.1538962154537993</v>
+        <v>0.2139313869052994</v>
       </c>
       <c r="N17" s="17" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="O17" s="17" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="P17" s="18">
-        <v>0.05593259931911281</v>
+        <v>0.1101859272146606</v>
       </c>
       <c r="Q17" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="R17" s="15" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="S17" s="16">
-        <v>0.154882674517742</v>
+        <v>0.09173394009831634</v>
       </c>
       <c r="T17" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="U17" s="17" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="V17" s="18">
-        <v>0.2917303773366727</v>
+        <v>0.1625945952836103</v>
       </c>
     </row>
     <row r="18" spans="1:22">
       <c r="A18" s="1"/>
       <c r="B18" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D18" s="10">
-        <v>0.1505536444536826</v>
+        <v>0.0879310177174988</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G18" s="12">
-        <v>0.026460857179454</v>
+        <v>0.09853456831250364</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J18" s="14">
-        <v>0.07835244941985345</v>
+        <v>0.1243464900873019</v>
       </c>
       <c r="K18" s="15" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="L18" s="15" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="M18" s="16">
-        <v>0.1421006539226223</v>
+        <v>0.1574954691188715</v>
       </c>
       <c r="N18" s="17" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="O18" s="17" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="P18" s="18">
-        <v>0.05494124543748962</v>
+        <v>0.1100578776840948</v>
       </c>
       <c r="Q18" s="15" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="R18" s="15" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="S18" s="16">
-        <v>0.06316624561074105</v>
+        <v>0.04211378157684734</v>
       </c>
       <c r="T18" s="17" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="U18" s="17" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="V18" s="18">
-        <v>0.105567828887357</v>
+        <v>0.1398484711814139</v>
       </c>
     </row>
     <row r="19" spans="1:22">
       <c r="A19" s="1"/>
       <c r="B19" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D19" s="10">
-        <v>0.05438206769808993</v>
+        <v>0.0525300210733301</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G19" s="12">
-        <v>0.02466868199880063</v>
+        <v>0.09629898229970971</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="J19" s="14">
-        <v>0.04939972259210003</v>
+        <v>0.1060353403575803</v>
       </c>
       <c r="K19" s="15" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="M19" s="16">
-        <v>0.09564947352725231</v>
+        <v>0.0676166400913904</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="O19" s="17" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="P19" s="18">
-        <v>0.01667226712768921</v>
+        <v>0.1048230125117821</v>
       </c>
       <c r="Q19" s="15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="R19" s="15" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="S19" s="16">
-        <v>0.03337189406657416</v>
+        <v>0.03954842646206794</v>
       </c>
       <c r="T19" s="17" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="U19" s="17" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="V19" s="18">
-        <v>0.03640298517399051</v>
+        <v>0.07959170762712155</v>
       </c>
     </row>
     <row r="20" spans="1:22">
       <c r="A20" s="1"/>
       <c r="B20" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D20" s="10">
-        <v>0.03788976491654274</v>
+        <v>0.03146419914196186</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>103</v>
+        <v>230</v>
       </c>
       <c r="G20" s="12">
-        <v>0.01239075614043313</v>
+        <v>0.02693030246291794</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="J20" s="14">
-        <v>0.02290263717500473</v>
+        <v>0.09608234375637947</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="L20" s="15" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="M20" s="16">
-        <v>0.09539911114614351</v>
+        <v>0.03747622629221283</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="O20" s="17" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="P20" s="18">
-        <v>0.01396830957029491</v>
+        <v>0.1028091649052724</v>
       </c>
       <c r="Q20" s="15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R20" s="15" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="S20" s="16">
-        <v>0.02647981733247263</v>
+        <v>0.02953372508226165</v>
       </c>
       <c r="T20" s="17" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="U20" s="17" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="V20" s="18">
-        <v>0.02707457648744899</v>
+        <v>0.07297275964797043</v>
       </c>
     </row>
   </sheetData>

</xml_diff>